<commit_message>
Fix: remove legacy sheet, fix dedup with leading-zero code normalization
</commit_message>
<xml_diff>
--- a/data/cot_master.xlsx
+++ b/data/cot_master.xlsx
@@ -7,12 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WTI_PHYSICAL_NYMEX" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="COT_Multi_Commodity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="COT_Multi_Commodity" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WTI_PHYSICAL_NYMEX'!$A$1:$T$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'COT_Multi_Commodity'!$A$1:$DV$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'COT_Multi_Commodity'!$A$1:$DV$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,2301 +418,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Report_Date_as_MM_DD_YYYY</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CFTC_Contract_Market_Code</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Open_Interest_All</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>NonComm_Positions_Long_All</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>NonComm_Positions_Short_All</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>NonComm_Postions_Spread_All</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Comm_Positions_Long_All</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Comm_Positions_Short_All</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Tot_Rept_Positions_Long_All</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Tot_Rept_Positions_Short_All</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>NonRept_Positions_Long_All</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>NonRept_Positions_Short_All</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Change_in_Open_Interest_All</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Change_in_NonComm_Long_All</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Change_in_NonComm_Short_All</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Pct_of_OI_NonComm_Long_All</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Pct_of_OI_NonComm_Short_All</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Pct_of_OI_Comm_Long_All</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Pct_of_OI_Comm_Short_All</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Contract_Units</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46028</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1968879</v>
-      </c>
-      <c r="D2" t="n">
-        <v>258956</v>
-      </c>
-      <c r="E2" t="n">
-        <v>201604</v>
-      </c>
-      <c r="F2" t="n">
-        <v>811995</v>
-      </c>
-      <c r="G2" t="n">
-        <v>829757</v>
-      </c>
-      <c r="H2" t="n">
-        <v>900523</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1900708</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1914122</v>
-      </c>
-      <c r="K2" t="n">
-        <v>68171</v>
-      </c>
-      <c r="L2" t="n">
-        <v>54757</v>
-      </c>
-      <c r="M2" t="n">
-        <v>70622</v>
-      </c>
-      <c r="N2" t="n">
-        <v>-2439</v>
-      </c>
-      <c r="O2" t="n">
-        <v>4800</v>
-      </c>
-      <c r="P2" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="R2" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46035</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2018789</v>
-      </c>
-      <c r="D3" t="n">
-        <v>286136</v>
-      </c>
-      <c r="E3" t="n">
-        <v>228008</v>
-      </c>
-      <c r="F3" t="n">
-        <v>812215</v>
-      </c>
-      <c r="G3" t="n">
-        <v>855313</v>
-      </c>
-      <c r="H3" t="n">
-        <v>920763</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1953664</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1960986</v>
-      </c>
-      <c r="K3" t="n">
-        <v>65125</v>
-      </c>
-      <c r="L3" t="n">
-        <v>57803</v>
-      </c>
-      <c r="M3" t="n">
-        <v>49910</v>
-      </c>
-      <c r="N3" t="n">
-        <v>27180</v>
-      </c>
-      <c r="O3" t="n">
-        <v>26404</v>
-      </c>
-      <c r="P3" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="R3" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="S3" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46042</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1964359</v>
-      </c>
-      <c r="D4" t="n">
-        <v>284809</v>
-      </c>
-      <c r="E4" t="n">
-        <v>206017</v>
-      </c>
-      <c r="F4" t="n">
-        <v>790703</v>
-      </c>
-      <c r="G4" t="n">
-        <v>821803</v>
-      </c>
-      <c r="H4" t="n">
-        <v>918850</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1897315</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1915570</v>
-      </c>
-      <c r="K4" t="n">
-        <v>67044</v>
-      </c>
-      <c r="L4" t="n">
-        <v>48789</v>
-      </c>
-      <c r="M4" t="n">
-        <v>-54430</v>
-      </c>
-      <c r="N4" t="n">
-        <v>-1327</v>
-      </c>
-      <c r="O4" t="n">
-        <v>-21991</v>
-      </c>
-      <c r="P4" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="R4" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="S4" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46049</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2035649</v>
-      </c>
-      <c r="D5" t="n">
-        <v>295247</v>
-      </c>
-      <c r="E5" t="n">
-        <v>198265</v>
-      </c>
-      <c r="F5" t="n">
-        <v>831414</v>
-      </c>
-      <c r="G5" t="n">
-        <v>840875</v>
-      </c>
-      <c r="H5" t="n">
-        <v>955923</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1967536</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1985602</v>
-      </c>
-      <c r="K5" t="n">
-        <v>68113</v>
-      </c>
-      <c r="L5" t="n">
-        <v>50047</v>
-      </c>
-      <c r="M5" t="n">
-        <v>71290</v>
-      </c>
-      <c r="N5" t="n">
-        <v>10438</v>
-      </c>
-      <c r="O5" t="n">
-        <v>-7752</v>
-      </c>
-      <c r="P5" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="R5" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="S5" t="n">
-        <v>47</v>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46056</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2091314</v>
-      </c>
-      <c r="D6" t="n">
-        <v>315529</v>
-      </c>
-      <c r="E6" t="n">
-        <v>190964</v>
-      </c>
-      <c r="F6" t="n">
-        <v>825127</v>
-      </c>
-      <c r="G6" t="n">
-        <v>879932</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1032431</v>
-      </c>
-      <c r="I6" t="n">
-        <v>2020588</v>
-      </c>
-      <c r="J6" t="n">
-        <v>2048522</v>
-      </c>
-      <c r="K6" t="n">
-        <v>70726</v>
-      </c>
-      <c r="L6" t="n">
-        <v>42792</v>
-      </c>
-      <c r="M6" t="n">
-        <v>55665</v>
-      </c>
-      <c r="N6" t="n">
-        <v>20282</v>
-      </c>
-      <c r="O6" t="n">
-        <v>-7301</v>
-      </c>
-      <c r="P6" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="R6" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="S6" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46063</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2070538</v>
-      </c>
-      <c r="D7" t="n">
-        <v>320742</v>
-      </c>
-      <c r="E7" t="n">
-        <v>202928</v>
-      </c>
-      <c r="F7" t="n">
-        <v>818843</v>
-      </c>
-      <c r="G7" t="n">
-        <v>846948</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1002814</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1986533</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2024585</v>
-      </c>
-      <c r="K7" t="n">
-        <v>84005</v>
-      </c>
-      <c r="L7" t="n">
-        <v>45953</v>
-      </c>
-      <c r="M7" t="n">
-        <v>-20776</v>
-      </c>
-      <c r="N7" t="n">
-        <v>5213</v>
-      </c>
-      <c r="O7" t="n">
-        <v>11964</v>
-      </c>
-      <c r="P7" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="R7" t="n">
-        <v>40.9</v>
-      </c>
-      <c r="S7" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46070</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2087493</v>
-      </c>
-      <c r="D8" t="n">
-        <v>321645</v>
-      </c>
-      <c r="E8" t="n">
-        <v>180302</v>
-      </c>
-      <c r="F8" t="n">
-        <v>829347</v>
-      </c>
-      <c r="G8" t="n">
-        <v>855378</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1037007</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2006370</v>
-      </c>
-      <c r="J8" t="n">
-        <v>2046656</v>
-      </c>
-      <c r="K8" t="n">
-        <v>81123</v>
-      </c>
-      <c r="L8" t="n">
-        <v>40837</v>
-      </c>
-      <c r="M8" t="n">
-        <v>16955</v>
-      </c>
-      <c r="N8" t="n">
-        <v>903</v>
-      </c>
-      <c r="O8" t="n">
-        <v>-22626</v>
-      </c>
-      <c r="P8" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="R8" t="n">
-        <v>41</v>
-      </c>
-      <c r="S8" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46077</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2102705</v>
-      </c>
-      <c r="D9" t="n">
-        <v>352565</v>
-      </c>
-      <c r="E9" t="n">
-        <v>179853</v>
-      </c>
-      <c r="F9" t="n">
-        <v>821589</v>
-      </c>
-      <c r="G9" t="n">
-        <v>827868</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1044651</v>
-      </c>
-      <c r="I9" t="n">
-        <v>2002022</v>
-      </c>
-      <c r="J9" t="n">
-        <v>2046093</v>
-      </c>
-      <c r="K9" t="n">
-        <v>100683</v>
-      </c>
-      <c r="L9" t="n">
-        <v>56612</v>
-      </c>
-      <c r="M9" t="n">
-        <v>15212</v>
-      </c>
-      <c r="N9" t="n">
-        <v>30920</v>
-      </c>
-      <c r="O9" t="n">
-        <v>-449</v>
-      </c>
-      <c r="P9" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="R9" t="n">
-        <v>39.4</v>
-      </c>
-      <c r="S9" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46084</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2073033</v>
-      </c>
-      <c r="D10" t="n">
-        <v>355158</v>
-      </c>
-      <c r="E10" t="n">
-        <v>183008</v>
-      </c>
-      <c r="F10" t="n">
-        <v>785693</v>
-      </c>
-      <c r="G10" t="n">
-        <v>842957</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1065284</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1983808</v>
-      </c>
-      <c r="J10" t="n">
-        <v>2033985</v>
-      </c>
-      <c r="K10" t="n">
-        <v>89225</v>
-      </c>
-      <c r="L10" t="n">
-        <v>39048</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-29672</v>
-      </c>
-      <c r="N10" t="n">
-        <v>2593</v>
-      </c>
-      <c r="O10" t="n">
-        <v>3155</v>
-      </c>
-      <c r="P10" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="R10" t="n">
-        <v>40.7</v>
-      </c>
-      <c r="S10" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>46091</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2051321</v>
-      </c>
-      <c r="D11" t="n">
-        <v>394651</v>
-      </c>
-      <c r="E11" t="n">
-        <v>166636</v>
-      </c>
-      <c r="F11" t="n">
-        <v>740683</v>
-      </c>
-      <c r="G11" t="n">
-        <v>827233</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1103680</v>
-      </c>
-      <c r="I11" t="n">
-        <v>1962567</v>
-      </c>
-      <c r="J11" t="n">
-        <v>2010999</v>
-      </c>
-      <c r="K11" t="n">
-        <v>88754</v>
-      </c>
-      <c r="L11" t="n">
-        <v>40322</v>
-      </c>
-      <c r="M11" t="n">
-        <v>-21712</v>
-      </c>
-      <c r="N11" t="n">
-        <v>39493</v>
-      </c>
-      <c r="O11" t="n">
-        <v>-16372</v>
-      </c>
-      <c r="P11" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="R11" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="S11" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>46098</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2081576</v>
-      </c>
-      <c r="D12" t="n">
-        <v>385768</v>
-      </c>
-      <c r="E12" t="n">
-        <v>167080</v>
-      </c>
-      <c r="F12" t="n">
-        <v>741925</v>
-      </c>
-      <c r="G12" t="n">
-        <v>857135</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1119764</v>
-      </c>
-      <c r="I12" t="n">
-        <v>1984828</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2028769</v>
-      </c>
-      <c r="K12" t="n">
-        <v>96748</v>
-      </c>
-      <c r="L12" t="n">
-        <v>52807</v>
-      </c>
-      <c r="M12" t="n">
-        <v>30255</v>
-      </c>
-      <c r="N12" t="n">
-        <v>-8883</v>
-      </c>
-      <c r="O12" t="n">
-        <v>444</v>
-      </c>
-      <c r="P12" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>8</v>
-      </c>
-      <c r="R12" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="S12" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>46105</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>2002065</v>
-      </c>
-      <c r="D13" t="n">
-        <v>376150</v>
-      </c>
-      <c r="E13" t="n">
-        <v>142530</v>
-      </c>
-      <c r="F13" t="n">
-        <v>708202</v>
-      </c>
-      <c r="G13" t="n">
-        <v>841200</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1108210</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1925552</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1958942</v>
-      </c>
-      <c r="K13" t="n">
-        <v>76513</v>
-      </c>
-      <c r="L13" t="n">
-        <v>43123</v>
-      </c>
-      <c r="M13" t="n">
-        <v>-79511</v>
-      </c>
-      <c r="N13" t="n">
-        <v>-9618</v>
-      </c>
-      <c r="O13" t="n">
-        <v>-24550</v>
-      </c>
-      <c r="P13" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="R13" t="n">
-        <v>42</v>
-      </c>
-      <c r="S13" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>46112</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>2030970</v>
-      </c>
-      <c r="D14" t="n">
-        <v>378087</v>
-      </c>
-      <c r="E14" t="n">
-        <v>164599</v>
-      </c>
-      <c r="F14" t="n">
-        <v>706316</v>
-      </c>
-      <c r="G14" t="n">
-        <v>870799</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1115890</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1955202</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1986805</v>
-      </c>
-      <c r="K14" t="n">
-        <v>75768</v>
-      </c>
-      <c r="L14" t="n">
-        <v>44165</v>
-      </c>
-      <c r="M14" t="n">
-        <v>28905</v>
-      </c>
-      <c r="N14" t="n">
-        <v>1937</v>
-      </c>
-      <c r="O14" t="n">
-        <v>22069</v>
-      </c>
-      <c r="P14" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="R14" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="S14" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46119</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2037857</v>
-      </c>
-      <c r="D15" t="n">
-        <v>381615</v>
-      </c>
-      <c r="E15" t="n">
-        <v>179462</v>
-      </c>
-      <c r="F15" t="n">
-        <v>690993</v>
-      </c>
-      <c r="G15" t="n">
-        <v>883576</v>
-      </c>
-      <c r="H15" t="n">
-        <v>1114042</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1956184</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1984497</v>
-      </c>
-      <c r="K15" t="n">
-        <v>81673</v>
-      </c>
-      <c r="L15" t="n">
-        <v>53360</v>
-      </c>
-      <c r="M15" t="n">
-        <v>6887</v>
-      </c>
-      <c r="N15" t="n">
-        <v>3528</v>
-      </c>
-      <c r="O15" t="n">
-        <v>14863</v>
-      </c>
-      <c r="P15" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="R15" t="n">
-        <v>43.4</v>
-      </c>
-      <c r="S15" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>46126</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>2094492</v>
-      </c>
-      <c r="D16" t="n">
-        <v>390468</v>
-      </c>
-      <c r="E16" t="n">
-        <v>183927</v>
-      </c>
-      <c r="F16" t="n">
-        <v>730854</v>
-      </c>
-      <c r="G16" t="n">
-        <v>891010</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1137945</v>
-      </c>
-      <c r="I16" t="n">
-        <v>2012332</v>
-      </c>
-      <c r="J16" t="n">
-        <v>2052726</v>
-      </c>
-      <c r="K16" t="n">
-        <v>82160</v>
-      </c>
-      <c r="L16" t="n">
-        <v>41766</v>
-      </c>
-      <c r="M16" t="n">
-        <v>56635</v>
-      </c>
-      <c r="N16" t="n">
-        <v>8853</v>
-      </c>
-      <c r="O16" t="n">
-        <v>4465</v>
-      </c>
-      <c r="P16" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="R16" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="S16" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>1984747</v>
-      </c>
-      <c r="D17" t="n">
-        <v>380020</v>
-      </c>
-      <c r="E17" t="n">
-        <v>187718</v>
-      </c>
-      <c r="F17" t="n">
-        <v>655341</v>
-      </c>
-      <c r="G17" t="n">
-        <v>873316</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1100027</v>
-      </c>
-      <c r="I17" t="n">
-        <v>1908677</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1943086</v>
-      </c>
-      <c r="K17" t="n">
-        <v>76070</v>
-      </c>
-      <c r="L17" t="n">
-        <v>41661</v>
-      </c>
-      <c r="M17" t="n">
-        <v>-109745</v>
-      </c>
-      <c r="N17" t="n">
-        <v>-10448</v>
-      </c>
-      <c r="O17" t="n">
-        <v>3791</v>
-      </c>
-      <c r="P17" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="R17" t="n">
-        <v>44</v>
-      </c>
-      <c r="S17" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>46140</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2017038</v>
-      </c>
-      <c r="D18" t="n">
-        <v>390683</v>
-      </c>
-      <c r="E18" t="n">
-        <v>198772</v>
-      </c>
-      <c r="F18" t="n">
-        <v>660076</v>
-      </c>
-      <c r="G18" t="n">
-        <v>890950</v>
-      </c>
-      <c r="H18" t="n">
-        <v>1110604</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1941709</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1969452</v>
-      </c>
-      <c r="K18" t="n">
-        <v>75329</v>
-      </c>
-      <c r="L18" t="n">
-        <v>47586</v>
-      </c>
-      <c r="M18" t="n">
-        <v>32291</v>
-      </c>
-      <c r="N18" t="n">
-        <v>10663</v>
-      </c>
-      <c r="O18" t="n">
-        <v>11054</v>
-      </c>
-      <c r="P18" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="R18" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="S18" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>46147</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2067827</v>
-      </c>
-      <c r="D19" t="n">
-        <v>381542</v>
-      </c>
-      <c r="E19" t="n">
-        <v>202756</v>
-      </c>
-      <c r="F19" t="n">
-        <v>673689</v>
-      </c>
-      <c r="G19" t="n">
-        <v>933442</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1139592</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1988673</v>
-      </c>
-      <c r="J19" t="n">
-        <v>2016037</v>
-      </c>
-      <c r="K19" t="n">
-        <v>79154</v>
-      </c>
-      <c r="L19" t="n">
-        <v>51790</v>
-      </c>
-      <c r="M19" t="n">
-        <v>50789</v>
-      </c>
-      <c r="N19" t="n">
-        <v>-9141</v>
-      </c>
-      <c r="O19" t="n">
-        <v>3984</v>
-      </c>
-      <c r="P19" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="R19" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="S19" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>46154</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>2081927</v>
-      </c>
-      <c r="D20" t="n">
-        <v>371491</v>
-      </c>
-      <c r="E20" t="n">
-        <v>201614</v>
-      </c>
-      <c r="F20" t="n">
-        <v>669802</v>
-      </c>
-      <c r="G20" t="n">
-        <v>958509</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1154643</v>
-      </c>
-      <c r="I20" t="n">
-        <v>1999802</v>
-      </c>
-      <c r="J20" t="n">
-        <v>2026059</v>
-      </c>
-      <c r="K20" t="n">
-        <v>82125</v>
-      </c>
-      <c r="L20" t="n">
-        <v>55868</v>
-      </c>
-      <c r="M20" t="n">
-        <v>14100</v>
-      </c>
-      <c r="N20" t="n">
-        <v>-10051</v>
-      </c>
-      <c r="O20" t="n">
-        <v>-1142</v>
-      </c>
-      <c r="P20" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="R20" t="n">
-        <v>46</v>
-      </c>
-      <c r="S20" t="n">
-        <v>55.5</v>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46161</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>2002950</v>
-      </c>
-      <c r="D21" t="n">
-        <v>384294</v>
-      </c>
-      <c r="E21" t="n">
-        <v>211714</v>
-      </c>
-      <c r="F21" t="n">
-        <v>639186</v>
-      </c>
-      <c r="G21" t="n">
-        <v>900625</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1101034</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1924105</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1951934</v>
-      </c>
-      <c r="K21" t="n">
-        <v>78845</v>
-      </c>
-      <c r="L21" t="n">
-        <v>51016</v>
-      </c>
-      <c r="M21" t="n">
-        <v>-78977</v>
-      </c>
-      <c r="N21" t="n">
-        <v>12803</v>
-      </c>
-      <c r="O21" t="n">
-        <v>10100</v>
-      </c>
-      <c r="P21" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="R21" t="n">
-        <v>45</v>
-      </c>
-      <c r="S21" t="n">
-        <v>55</v>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>46168</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2003795</v>
-      </c>
-      <c r="D22" t="n">
-        <v>378088</v>
-      </c>
-      <c r="E22" t="n">
-        <v>217090</v>
-      </c>
-      <c r="F22" t="n">
-        <v>641932</v>
-      </c>
-      <c r="G22" t="n">
-        <v>900997</v>
-      </c>
-      <c r="H22" t="n">
-        <v>1096470</v>
-      </c>
-      <c r="I22" t="n">
-        <v>1921017</v>
-      </c>
-      <c r="J22" t="n">
-        <v>1955492</v>
-      </c>
-      <c r="K22" t="n">
-        <v>82778</v>
-      </c>
-      <c r="L22" t="n">
-        <v>48303</v>
-      </c>
-      <c r="M22" t="n">
-        <v>845</v>
-      </c>
-      <c r="N22" t="n">
-        <v>-6206</v>
-      </c>
-      <c r="O22" t="n">
-        <v>5376</v>
-      </c>
-      <c r="P22" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="R22" t="n">
-        <v>45</v>
-      </c>
-      <c r="S22" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>46175</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>2025180</v>
-      </c>
-      <c r="D23" t="n">
-        <v>383310</v>
-      </c>
-      <c r="E23" t="n">
-        <v>227436</v>
-      </c>
-      <c r="F23" t="n">
-        <v>637536</v>
-      </c>
-      <c r="G23" t="n">
-        <v>918113</v>
-      </c>
-      <c r="H23" t="n">
-        <v>1106222</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1938959</v>
-      </c>
-      <c r="J23" t="n">
-        <v>1971194</v>
-      </c>
-      <c r="K23" t="n">
-        <v>86221</v>
-      </c>
-      <c r="L23" t="n">
-        <v>53986</v>
-      </c>
-      <c r="M23" t="n">
-        <v>21385</v>
-      </c>
-      <c r="N23" t="n">
-        <v>5222</v>
-      </c>
-      <c r="O23" t="n">
-        <v>10346</v>
-      </c>
-      <c r="P23" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="R23" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="S23" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>2006635</v>
-      </c>
-      <c r="D24" t="n">
-        <v>360524</v>
-      </c>
-      <c r="E24" t="n">
-        <v>230223</v>
-      </c>
-      <c r="F24" t="n">
-        <v>636781</v>
-      </c>
-      <c r="G24" t="n">
-        <v>919786</v>
-      </c>
-      <c r="H24" t="n">
-        <v>1090512</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1917091</v>
-      </c>
-      <c r="J24" t="n">
-        <v>1957516</v>
-      </c>
-      <c r="K24" t="n">
-        <v>89544</v>
-      </c>
-      <c r="L24" t="n">
-        <v>49119</v>
-      </c>
-      <c r="M24" t="n">
-        <v>-18545</v>
-      </c>
-      <c r="N24" t="n">
-        <v>-22786</v>
-      </c>
-      <c r="O24" t="n">
-        <v>2787</v>
-      </c>
-      <c r="P24" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="R24" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="S24" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>46189</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>2007709</v>
-      </c>
-      <c r="D25" t="n">
-        <v>361004</v>
-      </c>
-      <c r="E25" t="n">
-        <v>236521</v>
-      </c>
-      <c r="F25" t="n">
-        <v>642134</v>
-      </c>
-      <c r="G25" t="n">
-        <v>916343</v>
-      </c>
-      <c r="H25" t="n">
-        <v>1081682</v>
-      </c>
-      <c r="I25" t="n">
-        <v>1919481</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1960337</v>
-      </c>
-      <c r="K25" t="n">
-        <v>88228</v>
-      </c>
-      <c r="L25" t="n">
-        <v>47372</v>
-      </c>
-      <c r="M25" t="n">
-        <v>1074</v>
-      </c>
-      <c r="N25" t="n">
-        <v>480</v>
-      </c>
-      <c r="O25" t="n">
-        <v>6298</v>
-      </c>
-      <c r="P25" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="R25" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="S25" t="n">
-        <v>53.9</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>46196</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>1911877</v>
-      </c>
-      <c r="D26" t="n">
-        <v>350026</v>
-      </c>
-      <c r="E26" t="n">
-        <v>235393</v>
-      </c>
-      <c r="F26" t="n">
-        <v>602418</v>
-      </c>
-      <c r="G26" t="n">
-        <v>878059</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1030665</v>
-      </c>
-      <c r="I26" t="n">
-        <v>1830503</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1868476</v>
-      </c>
-      <c r="K26" t="n">
-        <v>81374</v>
-      </c>
-      <c r="L26" t="n">
-        <v>43401</v>
-      </c>
-      <c r="M26" t="n">
-        <v>-95832</v>
-      </c>
-      <c r="N26" t="n">
-        <v>-10978</v>
-      </c>
-      <c r="O26" t="n">
-        <v>-1128</v>
-      </c>
-      <c r="P26" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="R26" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="S26" t="n">
-        <v>53.9</v>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1914443</v>
-      </c>
-      <c r="D27" t="n">
-        <v>340698</v>
-      </c>
-      <c r="E27" t="n">
-        <v>230167</v>
-      </c>
-      <c r="F27" t="n">
-        <v>594641</v>
-      </c>
-      <c r="G27" t="n">
-        <v>902424</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1042572</v>
-      </c>
-      <c r="I27" t="n">
-        <v>1837763</v>
-      </c>
-      <c r="J27" t="n">
-        <v>1867380</v>
-      </c>
-      <c r="K27" t="n">
-        <v>76680</v>
-      </c>
-      <c r="L27" t="n">
-        <v>47063</v>
-      </c>
-      <c r="M27" t="n">
-        <v>2566</v>
-      </c>
-      <c r="N27" t="n">
-        <v>-9328</v>
-      </c>
-      <c r="O27" t="n">
-        <v>-5226</v>
-      </c>
-      <c r="P27" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>12</v>
-      </c>
-      <c r="R27" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="S27" t="n">
-        <v>54.5</v>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>46210</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>1905761</v>
-      </c>
-      <c r="D28" t="n">
-        <v>317773</v>
-      </c>
-      <c r="E28" t="n">
-        <v>242024</v>
-      </c>
-      <c r="F28" t="n">
-        <v>584653</v>
-      </c>
-      <c r="G28" t="n">
-        <v>924510</v>
-      </c>
-      <c r="H28" t="n">
-        <v>1029132</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1826936</v>
-      </c>
-      <c r="J28" t="n">
-        <v>1855809</v>
-      </c>
-      <c r="K28" t="n">
-        <v>78825</v>
-      </c>
-      <c r="L28" t="n">
-        <v>49952</v>
-      </c>
-      <c r="M28" t="n">
-        <v>-8682</v>
-      </c>
-      <c r="N28" t="n">
-        <v>-22925</v>
-      </c>
-      <c r="O28" t="n">
-        <v>11857</v>
-      </c>
-      <c r="P28" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="R28" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="S28" t="n">
-        <v>54</v>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>1875496</v>
-      </c>
-      <c r="D29" t="n">
-        <v>302429</v>
-      </c>
-      <c r="E29" t="n">
-        <v>239746</v>
-      </c>
-      <c r="F29" t="n">
-        <v>576997</v>
-      </c>
-      <c r="G29" t="n">
-        <v>923364</v>
-      </c>
-      <c r="H29" t="n">
-        <v>1008452</v>
-      </c>
-      <c r="I29" t="n">
-        <v>1802790</v>
-      </c>
-      <c r="J29" t="n">
-        <v>1825195</v>
-      </c>
-      <c r="K29" t="n">
-        <v>72706</v>
-      </c>
-      <c r="L29" t="n">
-        <v>50301</v>
-      </c>
-      <c r="M29" t="n">
-        <v>-30265</v>
-      </c>
-      <c r="N29" t="n">
-        <v>-15344</v>
-      </c>
-      <c r="O29" t="n">
-        <v>-2278</v>
-      </c>
-      <c r="P29" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="R29" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="S29" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>1864487</v>
-      </c>
-      <c r="D30" t="n">
-        <v>310182</v>
-      </c>
-      <c r="E30" t="n">
-        <v>228493</v>
-      </c>
-      <c r="F30" t="n">
-        <v>580934</v>
-      </c>
-      <c r="G30" t="n">
-        <v>896294</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1004895</v>
-      </c>
-      <c r="I30" t="n">
-        <v>1787410</v>
-      </c>
-      <c r="J30" t="n">
-        <v>1814322</v>
-      </c>
-      <c r="K30" t="n">
-        <v>77077</v>
-      </c>
-      <c r="L30" t="n">
-        <v>50165</v>
-      </c>
-      <c r="M30" t="n">
-        <v>-11009</v>
-      </c>
-      <c r="N30" t="n">
-        <v>7753</v>
-      </c>
-      <c r="O30" t="n">
-        <v>-11253</v>
-      </c>
-      <c r="P30" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="R30" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="S30" t="n">
-        <v>53.9</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>46231</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>1859795</v>
-      </c>
-      <c r="D31" t="n">
-        <v>314992</v>
-      </c>
-      <c r="E31" t="n">
-        <v>194884</v>
-      </c>
-      <c r="F31" t="n">
-        <v>595417</v>
-      </c>
-      <c r="G31" t="n">
-        <v>871589</v>
-      </c>
-      <c r="H31" t="n">
-        <v>1030411</v>
-      </c>
-      <c r="I31" t="n">
-        <v>1781998</v>
-      </c>
-      <c r="J31" t="n">
-        <v>1820712</v>
-      </c>
-      <c r="K31" t="n">
-        <v>77797</v>
-      </c>
-      <c r="L31" t="n">
-        <v>39083</v>
-      </c>
-      <c r="M31" t="n">
-        <v>-4692</v>
-      </c>
-      <c r="N31" t="n">
-        <v>4810</v>
-      </c>
-      <c r="O31" t="n">
-        <v>-33609</v>
-      </c>
-      <c r="P31" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="R31" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="S31" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="n">
-        <v>46238</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>1886816</v>
-      </c>
-      <c r="D32" t="n">
-        <v>308841</v>
-      </c>
-      <c r="E32" t="n">
-        <v>196398</v>
-      </c>
-      <c r="F32" t="n">
-        <v>610139</v>
-      </c>
-      <c r="G32" t="n">
-        <v>887525</v>
-      </c>
-      <c r="H32" t="n">
-        <v>1041300</v>
-      </c>
-      <c r="I32" t="n">
-        <v>1806505</v>
-      </c>
-      <c r="J32" t="n">
-        <v>1847837</v>
-      </c>
-      <c r="K32" t="n">
-        <v>80311</v>
-      </c>
-      <c r="L32" t="n">
-        <v>38979</v>
-      </c>
-      <c r="M32" t="n">
-        <v>27021</v>
-      </c>
-      <c r="N32" t="n">
-        <v>-6151</v>
-      </c>
-      <c r="O32" t="n">
-        <v>1514</v>
-      </c>
-      <c r="P32" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="R32" t="n">
-        <v>47</v>
-      </c>
-      <c r="S32" t="n">
-        <v>55.2</v>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>46245</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>1892429</v>
-      </c>
-      <c r="D33" t="n">
-        <v>314846</v>
-      </c>
-      <c r="E33" t="n">
-        <v>215650</v>
-      </c>
-      <c r="F33" t="n">
-        <v>604890</v>
-      </c>
-      <c r="G33" t="n">
-        <v>897344</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1026981</v>
-      </c>
-      <c r="I33" t="n">
-        <v>1817080</v>
-      </c>
-      <c r="J33" t="n">
-        <v>1847521</v>
-      </c>
-      <c r="K33" t="n">
-        <v>75349</v>
-      </c>
-      <c r="L33" t="n">
-        <v>44908</v>
-      </c>
-      <c r="M33" t="n">
-        <v>5613</v>
-      </c>
-      <c r="N33" t="n">
-        <v>6005</v>
-      </c>
-      <c r="O33" t="n">
-        <v>19252</v>
-      </c>
-      <c r="P33" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="R33" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="S33" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>46252</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>067651</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>1888960</v>
-      </c>
-      <c r="D34" t="n">
-        <v>320159</v>
-      </c>
-      <c r="E34" t="n">
-        <v>198069</v>
-      </c>
-      <c r="F34" t="n">
-        <v>598872</v>
-      </c>
-      <c r="G34" t="n">
-        <v>894821</v>
-      </c>
-      <c r="H34" t="n">
-        <v>1047908</v>
-      </c>
-      <c r="I34" t="n">
-        <v>1813852</v>
-      </c>
-      <c r="J34" t="n">
-        <v>1844849</v>
-      </c>
-      <c r="K34" t="n">
-        <v>75108</v>
-      </c>
-      <c r="L34" t="n">
-        <v>44111</v>
-      </c>
-      <c r="M34" t="n">
-        <v>-3469</v>
-      </c>
-      <c r="N34" t="n">
-        <v>5313</v>
-      </c>
-      <c r="O34" t="n">
-        <v>-17581</v>
-      </c>
-      <c r="P34" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="R34" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="S34" t="n">
-        <v>55.5</v>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>(CONTRACTS OF 1,000 BARRELS)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:T34"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:DV49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>